<commit_message>
fix home equity assurance dists
</commit_message>
<xml_diff>
--- a/resources/NamingTable.xlsx
+++ b/resources/NamingTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mstern\Documents\GitHub\effective_property_tax\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4807894F-3467-40B3-BE4F-0973AD83B059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F9D190-9BFE-45A7-AB7D-1B8D31AC050C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13230" uniqueCount="5832">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13233" uniqueCount="5833">
   <si>
     <t>County</t>
   </si>
@@ -17533,6 +17533,9 @@
   </si>
   <si>
     <t>154SSA</t>
+  </si>
+  <si>
+    <t>Home Equity Assurance District</t>
   </si>
 </sst>
 </file>
@@ -23945,6 +23948,9 @@
       <c r="D349">
         <v>110040000</v>
       </c>
+      <c r="E349" t="s">
+        <v>5832</v>
+      </c>
     </row>
     <row r="350" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
@@ -23959,6 +23965,9 @@
       <c r="D350">
         <v>110030000</v>
       </c>
+      <c r="E350" t="s">
+        <v>5832</v>
+      </c>
     </row>
     <row r="351" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
@@ -26131,6 +26140,9 @@
       </c>
       <c r="D478">
         <v>110020000</v>
+      </c>
+      <c r="E478" t="s">
+        <v>5832</v>
       </c>
     </row>
     <row r="479" spans="1:5" x14ac:dyDescent="0.3">
@@ -47980,7 +47992,7 @@
         <v>60</v>
       </c>
       <c r="F1798" t="str">
-        <f>C1798</f>
+        <f t="shared" ref="F1798:F1811" si="0">C1798</f>
         <v>VOLO SSA #9</v>
       </c>
     </row>
@@ -47998,7 +48010,7 @@
         <v>60</v>
       </c>
       <c r="F1799" t="str">
-        <f>C1799</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #8</v>
       </c>
     </row>
@@ -48016,7 +48028,7 @@
         <v>60</v>
       </c>
       <c r="F1800" t="str">
-        <f>C1800</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #6</v>
       </c>
     </row>
@@ -48034,7 +48046,7 @@
         <v>60</v>
       </c>
       <c r="F1801" t="str">
-        <f>C1801</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #5</v>
       </c>
     </row>
@@ -48052,7 +48064,7 @@
         <v>60</v>
       </c>
       <c r="F1802" t="str">
-        <f>C1802</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #4</v>
       </c>
     </row>
@@ -48070,7 +48082,7 @@
         <v>60</v>
       </c>
       <c r="F1803" t="str">
-        <f>C1803</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #3</v>
       </c>
     </row>
@@ -48088,7 +48100,7 @@
         <v>60</v>
       </c>
       <c r="F1804" t="str">
-        <f>C1804</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #2</v>
       </c>
     </row>
@@ -48106,7 +48118,7 @@
         <v>60</v>
       </c>
       <c r="F1805" t="str">
-        <f>C1805</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #18</v>
       </c>
     </row>
@@ -48124,7 +48136,7 @@
         <v>60</v>
       </c>
       <c r="F1806" t="str">
-        <f>C1806</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #17</v>
       </c>
     </row>
@@ -48142,7 +48154,7 @@
         <v>60</v>
       </c>
       <c r="F1807" t="str">
-        <f>C1807</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #16</v>
       </c>
     </row>
@@ -48160,7 +48172,7 @@
         <v>60</v>
       </c>
       <c r="F1808" t="str">
-        <f>C1808</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #15</v>
       </c>
     </row>
@@ -48178,7 +48190,7 @@
         <v>60</v>
       </c>
       <c r="F1809" t="str">
-        <f>C1809</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #14</v>
       </c>
     </row>
@@ -48196,7 +48208,7 @@
         <v>60</v>
       </c>
       <c r="F1810" t="str">
-        <f>C1810</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #11</v>
       </c>
     </row>
@@ -48214,7 +48226,7 @@
         <v>60</v>
       </c>
       <c r="F1811" t="str">
-        <f>C1811</f>
+        <f t="shared" si="0"/>
         <v>VOLO SSA #10</v>
       </c>
     </row>
@@ -48289,7 +48301,7 @@
         <v>60</v>
       </c>
       <c r="F1815" t="str">
-        <f>C1815</f>
+        <f t="shared" ref="F1815:F1820" si="1">C1815</f>
         <v>VERNON HILLS SSA #6</v>
       </c>
     </row>
@@ -48307,7 +48319,7 @@
         <v>60</v>
       </c>
       <c r="F1816" t="str">
-        <f>C1816</f>
+        <f t="shared" si="1"/>
         <v>VERNON HILLS SSA #5</v>
       </c>
     </row>
@@ -48325,7 +48337,7 @@
         <v>60</v>
       </c>
       <c r="F1817" t="str">
-        <f>C1817</f>
+        <f t="shared" si="1"/>
         <v>VERNON HILLS SSA #4</v>
       </c>
     </row>
@@ -48343,7 +48355,7 @@
         <v>60</v>
       </c>
       <c r="F1818" t="str">
-        <f>C1818</f>
+        <f t="shared" si="1"/>
         <v>VERNON HILLS SSA #3</v>
       </c>
     </row>
@@ -48361,7 +48373,7 @@
         <v>60</v>
       </c>
       <c r="F1819" t="str">
-        <f>C1819</f>
+        <f t="shared" si="1"/>
         <v>VERNON HILLS SSA #2</v>
       </c>
     </row>
@@ -48379,7 +48391,7 @@
         <v>60</v>
       </c>
       <c r="F1820" t="str">
-        <f>C1820</f>
+        <f t="shared" si="1"/>
         <v>VERNON HILLS SSA #1</v>
       </c>
     </row>
@@ -49388,7 +49400,7 @@
         <v>60</v>
       </c>
       <c r="F1879" t="str">
-        <f>C1879</f>
+        <f t="shared" ref="F1879:F1885" si="2">C1879</f>
         <v>ROUND LAKE SSA #4 - LAKEWOOD GROVE</v>
       </c>
     </row>
@@ -49406,7 +49418,7 @@
         <v>60</v>
       </c>
       <c r="F1880" t="str">
-        <f>C1880</f>
+        <f t="shared" si="2"/>
         <v>ROUND LAKE SSA #3 - LAKEWOOD GROVE</v>
       </c>
     </row>
@@ -49424,7 +49436,7 @@
         <v>60</v>
       </c>
       <c r="F1881" t="str">
-        <f>C1881</f>
+        <f t="shared" si="2"/>
         <v>ROUND LAKE SSA #2 - PW</v>
       </c>
     </row>
@@ -49442,7 +49454,7 @@
         <v>60</v>
       </c>
       <c r="F1882" t="str">
-        <f>C1882</f>
+        <f t="shared" si="2"/>
         <v>ROUND LAKE SSA #2 - LAKEWOOD GROVE</v>
       </c>
     </row>
@@ -49460,7 +49472,7 @@
         <v>60</v>
       </c>
       <c r="F1883" t="str">
-        <f>C1883</f>
+        <f t="shared" si="2"/>
         <v>ROUND LAKE SSA #1 - LAKEWOOD GROVE</v>
       </c>
     </row>
@@ -49478,7 +49490,7 @@
         <v>60</v>
       </c>
       <c r="F1884" t="str">
-        <f>C1884</f>
+        <f t="shared" si="2"/>
         <v>ROUND LAKE SSA #1 - BRIGHT MEADOWS</v>
       </c>
     </row>
@@ -49496,7 +49508,7 @@
         <v>60</v>
       </c>
       <c r="F1885" t="str">
-        <f>C1885</f>
+        <f t="shared" si="2"/>
         <v>ROUND LAKE SSA #1</v>
       </c>
     </row>
@@ -49759,7 +49771,7 @@
         <v>60</v>
       </c>
       <c r="F1899" t="str">
-        <f>C1899</f>
+        <f t="shared" ref="F1899:F1927" si="3">C1899</f>
         <v>RIVERWOODS SSA #9</v>
       </c>
     </row>
@@ -49777,7 +49789,7 @@
         <v>60</v>
       </c>
       <c r="F1900" t="str">
-        <f>C1900</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #8</v>
       </c>
     </row>
@@ -49795,7 +49807,7 @@
         <v>60</v>
       </c>
       <c r="F1901" t="str">
-        <f>C1901</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #7</v>
       </c>
     </row>
@@ -49813,7 +49825,7 @@
         <v>60</v>
       </c>
       <c r="F1902" t="str">
-        <f>C1902</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #6</v>
       </c>
     </row>
@@ -49831,7 +49843,7 @@
         <v>60</v>
       </c>
       <c r="F1903" t="str">
-        <f>C1903</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #5</v>
       </c>
     </row>
@@ -49849,7 +49861,7 @@
         <v>60</v>
       </c>
       <c r="F1904" t="str">
-        <f>C1904</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #4</v>
       </c>
     </row>
@@ -49867,7 +49879,7 @@
         <v>60</v>
       </c>
       <c r="F1905" t="str">
-        <f>C1905</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #32</v>
       </c>
     </row>
@@ -49885,7 +49897,7 @@
         <v>60</v>
       </c>
       <c r="F1906" t="str">
-        <f>C1906</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #31</v>
       </c>
     </row>
@@ -49903,7 +49915,7 @@
         <v>60</v>
       </c>
       <c r="F1907" t="str">
-        <f>C1907</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #30</v>
       </c>
     </row>
@@ -49921,7 +49933,7 @@
         <v>60</v>
       </c>
       <c r="F1908" t="str">
-        <f>C1908</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #3</v>
       </c>
     </row>
@@ -49939,7 +49951,7 @@
         <v>60</v>
       </c>
       <c r="F1909" t="str">
-        <f>C1909</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #29</v>
       </c>
     </row>
@@ -49957,7 +49969,7 @@
         <v>60</v>
       </c>
       <c r="F1910" t="str">
-        <f>C1910</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #28</v>
       </c>
     </row>
@@ -49975,7 +49987,7 @@
         <v>60</v>
       </c>
       <c r="F1911" t="str">
-        <f>C1911</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #27</v>
       </c>
     </row>
@@ -49993,7 +50005,7 @@
         <v>60</v>
       </c>
       <c r="F1912" t="str">
-        <f>C1912</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #26</v>
       </c>
     </row>
@@ -50011,7 +50023,7 @@
         <v>60</v>
       </c>
       <c r="F1913" t="str">
-        <f>C1913</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #25</v>
       </c>
     </row>
@@ -50029,7 +50041,7 @@
         <v>60</v>
       </c>
       <c r="F1914" t="str">
-        <f>C1914</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #24</v>
       </c>
     </row>
@@ -50047,7 +50059,7 @@
         <v>60</v>
       </c>
       <c r="F1915" t="str">
-        <f>C1915</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #23</v>
       </c>
     </row>
@@ -50065,7 +50077,7 @@
         <v>60</v>
       </c>
       <c r="F1916" t="str">
-        <f>C1916</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #22</v>
       </c>
     </row>
@@ -50083,7 +50095,7 @@
         <v>60</v>
       </c>
       <c r="F1917" t="str">
-        <f>C1917</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #21</v>
       </c>
     </row>
@@ -50101,7 +50113,7 @@
         <v>60</v>
       </c>
       <c r="F1918" t="str">
-        <f>C1918</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #20</v>
       </c>
     </row>
@@ -50119,7 +50131,7 @@
         <v>60</v>
       </c>
       <c r="F1919" t="str">
-        <f>C1919</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #19</v>
       </c>
     </row>
@@ -50137,7 +50149,7 @@
         <v>60</v>
       </c>
       <c r="F1920" t="str">
-        <f>C1920</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #18</v>
       </c>
     </row>
@@ -50155,7 +50167,7 @@
         <v>60</v>
       </c>
       <c r="F1921" t="str">
-        <f>C1921</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #17</v>
       </c>
     </row>
@@ -50173,7 +50185,7 @@
         <v>60</v>
       </c>
       <c r="F1922" t="str">
-        <f>C1922</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #16</v>
       </c>
     </row>
@@ -50191,7 +50203,7 @@
         <v>60</v>
       </c>
       <c r="F1923" t="str">
-        <f>C1923</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #15</v>
       </c>
     </row>
@@ -50209,7 +50221,7 @@
         <v>60</v>
       </c>
       <c r="F1924" t="str">
-        <f>C1924</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #14</v>
       </c>
     </row>
@@ -50227,7 +50239,7 @@
         <v>60</v>
       </c>
       <c r="F1925" t="str">
-        <f>C1925</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #12</v>
       </c>
     </row>
@@ -50245,7 +50257,7 @@
         <v>60</v>
       </c>
       <c r="F1926" t="str">
-        <f>C1926</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #11</v>
       </c>
     </row>
@@ -50263,7 +50275,7 @@
         <v>60</v>
       </c>
       <c r="F1927" t="str">
-        <f>C1927</f>
+        <f t="shared" si="3"/>
         <v>RIVERWOODS SSA #10</v>
       </c>
     </row>
@@ -50454,7 +50466,7 @@
         <v>60</v>
       </c>
       <c r="F1937" t="str">
-        <f>C1937</f>
+        <f t="shared" ref="F1937:F1945" si="4">C1937</f>
         <v>NORTH BARRINGTON SSA #7</v>
       </c>
     </row>
@@ -50472,7 +50484,7 @@
         <v>60</v>
       </c>
       <c r="F1938" t="str">
-        <f>C1938</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #6</v>
       </c>
     </row>
@@ -50490,7 +50502,7 @@
         <v>60</v>
       </c>
       <c r="F1939" t="str">
-        <f>C1939</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #5</v>
       </c>
     </row>
@@ -50508,7 +50520,7 @@
         <v>60</v>
       </c>
       <c r="F1940" t="str">
-        <f>C1940</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #18</v>
       </c>
     </row>
@@ -50526,7 +50538,7 @@
         <v>60</v>
       </c>
       <c r="F1941" t="str">
-        <f>C1941</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #18</v>
       </c>
     </row>
@@ -50544,7 +50556,7 @@
         <v>60</v>
       </c>
       <c r="F1942" t="str">
-        <f>C1942</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #17</v>
       </c>
     </row>
@@ -50562,7 +50574,7 @@
         <v>60</v>
       </c>
       <c r="F1943" t="str">
-        <f>C1943</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #15</v>
       </c>
     </row>
@@ -50580,7 +50592,7 @@
         <v>60</v>
       </c>
       <c r="F1944" t="str">
-        <f>C1944</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #14</v>
       </c>
     </row>
@@ -50598,7 +50610,7 @@
         <v>60</v>
       </c>
       <c r="F1945" t="str">
-        <f>C1945</f>
+        <f t="shared" si="4"/>
         <v>NORTH BARRINGTON SSA #13</v>
       </c>
     </row>
@@ -50787,7 +50799,7 @@
         <v>60</v>
       </c>
       <c r="F1955" t="str">
-        <f>C1955</f>
+        <f t="shared" ref="F1955:F1966" si="5">C1955</f>
         <v>METTAWA SSA #8Z</v>
       </c>
     </row>
@@ -50805,7 +50817,7 @@
         <v>60</v>
       </c>
       <c r="F1956" t="str">
-        <f>C1956</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8Y</v>
       </c>
     </row>
@@ -50823,7 +50835,7 @@
         <v>60</v>
       </c>
       <c r="F1957" t="str">
-        <f>C1957</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8X</v>
       </c>
     </row>
@@ -50841,7 +50853,7 @@
         <v>60</v>
       </c>
       <c r="F1958" t="str">
-        <f>C1958</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8W</v>
       </c>
     </row>
@@ -50859,7 +50871,7 @@
         <v>60</v>
       </c>
       <c r="F1959" t="str">
-        <f>C1959</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8V</v>
       </c>
     </row>
@@ -50877,7 +50889,7 @@
         <v>60</v>
       </c>
       <c r="F1960" t="str">
-        <f>C1960</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8U</v>
       </c>
     </row>
@@ -50895,7 +50907,7 @@
         <v>60</v>
       </c>
       <c r="F1961" t="str">
-        <f>C1961</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8T</v>
       </c>
     </row>
@@ -50913,7 +50925,7 @@
         <v>60</v>
       </c>
       <c r="F1962" t="str">
-        <f>C1962</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8S</v>
       </c>
     </row>
@@ -50931,7 +50943,7 @@
         <v>60</v>
       </c>
       <c r="F1963" t="str">
-        <f>C1963</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8R</v>
       </c>
     </row>
@@ -50949,7 +50961,7 @@
         <v>60</v>
       </c>
       <c r="F1964" t="str">
-        <f>C1964</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8Q</v>
       </c>
     </row>
@@ -50967,7 +50979,7 @@
         <v>60</v>
       </c>
       <c r="F1965" t="str">
-        <f>C1965</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8P</v>
       </c>
     </row>
@@ -50985,7 +50997,7 @@
         <v>60</v>
       </c>
       <c r="F1966" t="str">
-        <f>C1966</f>
+        <f t="shared" si="5"/>
         <v>METTAWA SSA #8O</v>
       </c>
     </row>
@@ -51510,7 +51522,7 @@
         <v>60</v>
       </c>
       <c r="F1996" t="str">
-        <f>C1996</f>
+        <f t="shared" ref="F1996:F2010" si="6">C1996</f>
         <v>METTAWA SSA #6Q</v>
       </c>
     </row>
@@ -51528,7 +51540,7 @@
         <v>60</v>
       </c>
       <c r="F1997" t="str">
-        <f>C1997</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6P</v>
       </c>
     </row>
@@ -51546,7 +51558,7 @@
         <v>60</v>
       </c>
       <c r="F1998" t="str">
-        <f>C1998</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6O</v>
       </c>
     </row>
@@ -51564,7 +51576,7 @@
         <v>60</v>
       </c>
       <c r="F1999" t="str">
-        <f>C1999</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6N</v>
       </c>
     </row>
@@ -51582,7 +51594,7 @@
         <v>60</v>
       </c>
       <c r="F2000" t="str">
-        <f>C2000</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6M</v>
       </c>
     </row>
@@ -51600,7 +51612,7 @@
         <v>60</v>
       </c>
       <c r="F2001" t="str">
-        <f>C2001</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6L</v>
       </c>
     </row>
@@ -51618,7 +51630,7 @@
         <v>60</v>
       </c>
       <c r="F2002" t="str">
-        <f>C2002</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6K</v>
       </c>
     </row>
@@ -51636,7 +51648,7 @@
         <v>60</v>
       </c>
       <c r="F2003" t="str">
-        <f>C2003</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6J</v>
       </c>
     </row>
@@ -51654,7 +51666,7 @@
         <v>60</v>
       </c>
       <c r="F2004" t="str">
-        <f>C2004</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6I</v>
       </c>
     </row>
@@ -51672,7 +51684,7 @@
         <v>60</v>
       </c>
       <c r="F2005" t="str">
-        <f>C2005</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6H</v>
       </c>
     </row>
@@ -51690,7 +51702,7 @@
         <v>60</v>
       </c>
       <c r="F2006" t="str">
-        <f>C2006</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6G</v>
       </c>
     </row>
@@ -51708,7 +51720,7 @@
         <v>60</v>
       </c>
       <c r="F2007" t="str">
-        <f>C2007</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6F</v>
       </c>
     </row>
@@ -51726,7 +51738,7 @@
         <v>60</v>
       </c>
       <c r="F2008" t="str">
-        <f>C2008</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6E</v>
       </c>
     </row>
@@ -51744,7 +51756,7 @@
         <v>60</v>
       </c>
       <c r="F2009" t="str">
-        <f>C2009</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6D</v>
       </c>
     </row>
@@ -51762,7 +51774,7 @@
         <v>60</v>
       </c>
       <c r="F2010" t="str">
-        <f>C2010</f>
+        <f t="shared" si="6"/>
         <v>METTAWA SSA #6C</v>
       </c>
     </row>

</xml_diff>